<commit_message>
docs: mise à jour Excel session 27 avril 2026
</commit_message>
<xml_diff>
--- a/Création Muse Switzerland Market Place .xlsx
+++ b/Création Muse Switzerland Market Place .xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0c987177a5198109/Desktop/DOSSIER DIVERS A TRIER/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0c987177a5198109/Desktop/ANTHROPIC/Muse Switzerland/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="283" documentId="8_{ACF85F94-045C-4991-B3D2-B847DC23EF8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04ADB493-0C11-4FAD-8CDB-DFA24879E853}"/>
+  <xr:revisionPtr revIDLastSave="356" documentId="8_{ACF85F94-045C-4991-B3D2-B847DC23EF8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4F83D19-EF5F-44D6-815D-5A679359E8B2}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{8BEFC220-E72D-4D45-B16E-ECB5CB17A6D0}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="112">
   <si>
     <t>Objectifs</t>
   </si>
@@ -244,6 +244,135 @@
   </si>
   <si>
     <t>ETAPE AVANCEMENT PROJET</t>
+  </si>
+  <si>
+    <t>Logo Ms dans le header Divi</t>
+  </si>
+  <si>
+    <t>Fond beige sur section chiffres clés</t>
+  </si>
+  <si>
+    <t>Réduire l'espace blanc entre les sections</t>
+  </si>
+  <si>
+    <t>Mettre le fond beige sur la section trust bar</t>
+  </si>
+  <si>
+    <t>Travailler sur le header (burger, logo centré, icônes)</t>
+  </si>
+  <si>
+    <t>Sauvegarder sur GitHub</t>
+  </si>
+  <si>
+    <t>Thème enfant Divi créé et activé CSS Muse Switzerland chargé  Menu nettoyé — Homme + Femme uniquement</t>
+  </si>
+  <si>
+    <t>Hero, citation, chiffres clés, catégories, trust bar, CTA vendeur, footer</t>
+  </si>
+  <si>
+    <t>HEADER</t>
+  </si>
+  <si>
+    <t>Logo Ms monogramme SVG 42px centré dans carré</t>
+  </si>
+  <si>
+    <t>Structure 3 colonnes : burger+nav gauche | logo centre | icônes droite</t>
+  </si>
+  <si>
+    <t>Burger ≡ avec menu overlay : Femme, Homme, Enfant, Accessoires, Mon compte, Vendre</t>
+  </si>
+  <si>
+    <t>Navigation : FEMME / HOMME en uppercase Jost 11px</t>
+  </si>
+  <si>
+    <t>Icônes droite : FR + loupe + compte + panier (SVG stroke 1.2px)</t>
+  </si>
+  <si>
+    <t>SECTION MOSAÏQUE</t>
+  </si>
+  <si>
+    <t>4 images pleine largeur entre header et hero</t>
+  </si>
+  <si>
+    <t>Texte "✦ Offre exclusive / Livraison gratuite dès CHF 150.–" en blanc</t>
+  </si>
+  <si>
+    <t>Images : vêtements femme / vêtements homme / bague dorée / sac cuir</t>
+  </si>
+  <si>
+    <t>HERO HOMEPAGE</t>
+  </si>
+  <si>
+    <t>Structure 3 colonnes : photo femme | texte centre | photo homme</t>
+  </si>
+  <si>
+    <t>3 boutons : DÉCOUVRIR LA COLLECTION (noir) / VENDRE MES ARTICLES (contour) / DEVENIR VENDEUR (contour rouge)</t>
+  </si>
+  <si>
+    <t>SECTIONS HOMEPAGE</t>
+  </si>
+  <si>
+    <t>Fond beige #F2EFE9 sur chiffres clés (320/12K+/CH)</t>
+  </si>
+  <si>
+    <t>Fond beige #F2EFE9 sur trust bar (4 colonnes avec ✦ rouge)</t>
+  </si>
+  <si>
+    <t>"PARCOURIR PAR / Catégories" agrandi (11px / 36px)</t>
+  </si>
+  <si>
+    <t>Fond beige sur section catégories</t>
+  </si>
+  <si>
+    <t>CTA vendeur pleine largeur fond noir #111110</t>
+  </si>
+  <si>
+    <t>Footer beige 4 colonnes + barre copyright noire avec badges STRIPE/TWINT/VISA/MASTERCARD</t>
+  </si>
+  <si>
+    <t>Suppression texte "Design de Elegant Themes"</t>
+  </si>
+  <si>
+    <t>PAGE FEMME</t>
+  </si>
+  <si>
+    <t>Bandeau hero : COLLECTION / Femme / « Parce que vous êtes toutes des muses » / 1 840 articles</t>
+  </si>
+  <si>
+    <t>Module Produits Woo ajouté — en cours de configuration (4 colonnes, ordre récent)</t>
+  </si>
+  <si>
+    <t>FICHIERS GITHUB</t>
+  </si>
+  <si>
+    <t>CLAUDE_INSTRUCTIONS.md — instructions complètes du projet</t>
+  </si>
+  <si>
+    <t>assets/css/muse-design-system.css — CSS complet</t>
+  </si>
+  <si>
+    <t>assets/js/muse-main.js — JS principal</t>
+  </si>
+  <si>
+    <t>assets/svg/muse-logo-monogram.svg — logo Ms</t>
+  </si>
+  <si>
+    <t>PROCHAINES ÉTAPES</t>
+  </si>
+  <si>
+    <t>Finir configuration module Produits Woo page Femme</t>
+  </si>
+  <si>
+    <t>Page Homme</t>
+  </si>
+  <si>
+    <t>Fiche produit avec badges état + "Fréquemment achetés ensemble"</t>
+  </si>
+  <si>
+    <t>Checkout avec TVA 7.7%</t>
+  </si>
+  <si>
+    <t>Mobile responsive</t>
   </si>
 </sst>
 </file>
@@ -477,7 +606,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
@@ -517,9 +646,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -535,7 +661,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -548,6 +673,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -901,55 +1029,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D75BACB6-41E5-4C7B-BA64-F2B8423A2BF6}">
-  <dimension ref="A1:N54"/>
+  <dimension ref="A1:N97"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="57.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="123" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.1796875" customWidth="1"/>
     <col min="3" max="3" width="17.7265625" style="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.26953125" customWidth="1"/>
     <col min="5" max="5" width="59.7265625" style="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="29.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="29.1796875" style="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="35" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
     </row>
     <row r="2" spans="1:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
+      <c r="A2" s="35"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="N3" s="26" t="s">
+      <c r="N3" s="25" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="35" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="36" t="s">
+      <c r="B4" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="36" t="s">
+      <c r="E4" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="25" t="s">
+      <c r="N4" s="24" t="s">
         <v>6</v>
       </c>
     </row>
@@ -960,13 +1088,13 @@
       <c r="B5" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="4"/>
       <c r="F5" s="5"/>
-      <c r="N5" s="25" t="s">
+      <c r="N5" s="24" t="s">
         <v>5</v>
       </c>
     </row>
@@ -977,13 +1105,13 @@
       <c r="B6" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="4"/>
       <c r="F6" s="5"/>
-      <c r="N6" s="25" t="s">
+      <c r="N6" s="24" t="s">
         <v>7</v>
       </c>
     </row>
@@ -994,13 +1122,13 @@
       <c r="B7" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="4"/>
       <c r="F7" s="5"/>
-      <c r="N7" s="25"/>
+      <c r="N7" s="24"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
@@ -1009,7 +1137,7 @@
       <c r="B8" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="3"/>
@@ -1023,7 +1151,7 @@
       <c r="B9" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="3"/>
@@ -1037,13 +1165,13 @@
       <c r="B10" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="4"/>
       <c r="F10" s="8"/>
-      <c r="N10" s="25"/>
+      <c r="N10" s="24"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
@@ -1052,7 +1180,7 @@
       <c r="B11" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C11" s="27" t="s">
+      <c r="C11" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="3"/>
@@ -1066,13 +1194,13 @@
       <c r="B12" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C12" s="27" t="s">
+      <c r="C12" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="4"/>
       <c r="F12" s="5"/>
-      <c r="N12" s="25"/>
+      <c r="N12" s="24"/>
     </row>
     <row r="13" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="16" t="s">
@@ -1081,12 +1209,12 @@
       <c r="B13" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C13" s="28" t="s">
+      <c r="C13" s="27" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="18"/>
       <c r="E13" s="19"/>
-      <c r="N13" s="25"/>
+      <c r="N13" s="24"/>
     </row>
     <row r="14" spans="1:14" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.4">
       <c r="A14" s="15" t="s">
@@ -1095,11 +1223,11 @@
       <c r="B14" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C14" s="27"/>
+      <c r="C14" s="26"/>
       <c r="D14" s="3"/>
       <c r="E14" s="4"/>
       <c r="F14" s="5"/>
-      <c r="N14" s="25"/>
+      <c r="N14" s="24"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
@@ -1108,7 +1236,7 @@
       <c r="B15" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D15" s="3"/>
@@ -1122,7 +1250,7 @@
       <c r="B16" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="3"/>
@@ -1137,7 +1265,7 @@
       <c r="B17" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D17" s="3"/>
@@ -1154,7 +1282,7 @@
       <c r="B18" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D18" s="3"/>
@@ -1169,7 +1297,7 @@
       <c r="B19" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C19" s="27" t="s">
+      <c r="C19" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="3"/>
@@ -1183,7 +1311,7 @@
       <c r="B20" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C20" s="27" t="s">
+      <c r="C20" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D20" s="3"/>
@@ -1199,7 +1327,7 @@
       <c r="B21" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C21" s="27" t="s">
+      <c r="C21" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="3"/>
@@ -1214,7 +1342,7 @@
       <c r="B22" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C22" s="27" t="s">
+      <c r="C22" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D22" s="3"/>
@@ -1228,7 +1356,7 @@
       <c r="B23" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C23" s="27" t="s">
+      <c r="C23" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D23" s="3"/>
@@ -1241,7 +1369,7 @@
       <c r="B24" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C24" s="27" t="s">
+      <c r="C24" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D24" s="3"/>
@@ -1255,7 +1383,7 @@
       <c r="B25" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C25" s="28" t="s">
+      <c r="C25" s="27" t="s">
         <v>7</v>
       </c>
       <c r="D25" s="18"/>
@@ -1268,7 +1396,7 @@
       <c r="B26" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="C26" s="27"/>
+      <c r="C26" s="26"/>
       <c r="D26" s="3"/>
       <c r="E26" s="4"/>
     </row>
@@ -1279,7 +1407,7 @@
       <c r="B27" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C27" s="27" t="s">
+      <c r="C27" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D27" s="3"/>
@@ -1293,7 +1421,7 @@
       <c r="B28" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C28" s="27" t="s">
+      <c r="C28" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D28" s="3"/>
@@ -1308,7 +1436,7 @@
       <c r="B29" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="C29" s="27" t="s">
+      <c r="C29" s="26" t="s">
         <v>5</v>
       </c>
       <c r="D29" s="3"/>
@@ -1319,7 +1447,7 @@
         <v>36</v>
       </c>
       <c r="B30" s="2"/>
-      <c r="C30" s="27" t="s">
+      <c r="C30" s="26" t="s">
         <v>5</v>
       </c>
       <c r="D30" s="3"/>
@@ -1334,7 +1462,7 @@
       <c r="B31" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C31" s="27" t="s">
+      <c r="C31" s="26" t="s">
         <v>7</v>
       </c>
       <c r="D31" s="3"/>
@@ -1347,7 +1475,7 @@
       <c r="B32" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C32" s="28" t="s">
+      <c r="C32" s="27" t="s">
         <v>7</v>
       </c>
       <c r="D32" s="18"/>
@@ -1358,7 +1486,7 @@
         <v>40</v>
       </c>
       <c r="B33" s="2"/>
-      <c r="C33" s="27"/>
+      <c r="C33" s="26"/>
       <c r="D33" s="3"/>
       <c r="E33" s="4"/>
     </row>
@@ -1366,54 +1494,90 @@
       <c r="A34" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B34" s="2"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="3"/>
+      <c r="B34" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C34" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="3">
+        <v>46136</v>
+      </c>
       <c r="E34" s="4"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B35" s="2"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="3"/>
+      <c r="B35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C35" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="3">
+        <v>46136</v>
+      </c>
       <c r="E35" s="4"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B36" s="2"/>
-      <c r="C36" s="27"/>
-      <c r="D36" s="3"/>
+      <c r="B36" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C36" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="3">
+        <v>46136</v>
+      </c>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B37" s="2"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="3"/>
+      <c r="B37" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C37" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="3">
+        <v>46136</v>
+      </c>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B38" s="2"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="14"/>
+      <c r="B38" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C38" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="3">
+        <v>46136</v>
+      </c>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B39" s="17"/>
-      <c r="C39" s="28"/>
-      <c r="D39" s="20"/>
+      <c r="B39" s="17" t="b">
+        <v>1</v>
+      </c>
+      <c r="C39" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="18">
+        <v>46136</v>
+      </c>
       <c r="E39" s="19"/>
     </row>
     <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.4">
@@ -1421,7 +1585,9 @@
         <v>47</v>
       </c>
       <c r="B40" s="2"/>
-      <c r="C40" s="27"/>
+      <c r="C40" s="27" t="s">
+        <v>7</v>
+      </c>
       <c r="D40" s="14"/>
       <c r="E40" s="4"/>
     </row>
@@ -1430,7 +1596,9 @@
         <v>48</v>
       </c>
       <c r="B41" s="2"/>
-      <c r="C41" s="27"/>
+      <c r="C41" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D41" s="14"/>
       <c r="E41" s="4"/>
     </row>
@@ -1439,7 +1607,9 @@
         <v>49</v>
       </c>
       <c r="B42" s="2"/>
-      <c r="C42" s="27"/>
+      <c r="C42" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D42" s="14"/>
       <c r="E42" s="4"/>
     </row>
@@ -1448,7 +1618,9 @@
         <v>50</v>
       </c>
       <c r="B43" s="2"/>
-      <c r="C43" s="27"/>
+      <c r="C43" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D43" s="14"/>
       <c r="E43" s="4"/>
     </row>
@@ -1456,8 +1628,12 @@
       <c r="A44" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B44" s="2"/>
-      <c r="C44" s="27"/>
+      <c r="B44" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C44" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D44" s="14"/>
       <c r="E44" s="4"/>
     </row>
@@ -1466,7 +1642,9 @@
         <v>52</v>
       </c>
       <c r="B45" s="2"/>
-      <c r="C45" s="27"/>
+      <c r="C45" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D45" s="14"/>
       <c r="E45" s="4"/>
     </row>
@@ -1475,72 +1653,661 @@
         <v>53</v>
       </c>
       <c r="B46" s="17"/>
-      <c r="C46" s="28"/>
+      <c r="C46" s="27" t="s">
+        <v>7</v>
+      </c>
       <c r="D46" s="20"/>
       <c r="E46" s="19"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47" s="1"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="27"/>
+    <row r="47" spans="1:5" ht="16" x14ac:dyDescent="0.4">
+      <c r="A47" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="B47" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C47" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D47" s="14"/>
       <c r="E47" s="4"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" s="1"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="27"/>
+      <c r="A48" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B48" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C48" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D48" s="14"/>
       <c r="E48" s="4"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="1"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="27"/>
+      <c r="A49" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B49" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C49" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D49" s="14"/>
       <c r="E49" s="4"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="1"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="27"/>
+      <c r="A50" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B50" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C50" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D50" s="14"/>
       <c r="E50" s="4"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="1"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="27"/>
+      <c r="A51" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B51" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C51" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D51" s="14"/>
       <c r="E51" s="4"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="1"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="27"/>
+      <c r="A52" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B52" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C52" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D52" s="14"/>
       <c r="E52" s="4"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A53" s="1"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="27"/>
+      <c r="A53" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B53" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C53" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D53" s="14"/>
       <c r="E53" s="4"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A54" s="1"/>
+      <c r="A54" s="1" t="s">
+        <v>76</v>
+      </c>
       <c r="B54" s="2"/>
-      <c r="C54" s="27"/>
+      <c r="C54" s="26" t="s">
+        <v>7</v>
+      </c>
       <c r="D54" s="14"/>
       <c r="E54" s="4"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" s="16"/>
+      <c r="B55" s="17"/>
+      <c r="C55" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55" s="20"/>
+      <c r="E55" s="19"/>
+    </row>
+    <row r="56" spans="1:5" ht="16" x14ac:dyDescent="0.4">
+      <c r="A56" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="B56" s="2"/>
+      <c r="C56" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E56" s="4"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A57" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B57" s="2"/>
+      <c r="C57" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E57" s="4"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B58" s="2"/>
+      <c r="C58" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D58" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E58" s="4"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A59" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B59" s="2"/>
+      <c r="C59" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E59" s="4"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B60" s="2"/>
+      <c r="C60" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E60" s="4"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B61" s="2"/>
+      <c r="C61" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D61" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E61" s="4"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" s="16"/>
+      <c r="B62" s="17"/>
+      <c r="C62" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62" s="18">
+        <v>46139</v>
+      </c>
+      <c r="E62" s="19"/>
+    </row>
+    <row r="63" spans="1:5" ht="16" x14ac:dyDescent="0.4">
+      <c r="A63" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B63" s="2"/>
+      <c r="C63" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D63" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E63" s="4"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A64" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B64" s="2"/>
+      <c r="C64" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E64" s="4"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A65" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B65" s="2"/>
+      <c r="C65" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E65" s="4"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A66" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B66" s="2"/>
+      <c r="C66" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E66" s="4"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A67" s="1"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E67" s="4"/>
+    </row>
+    <row r="68" spans="1:5" ht="16" x14ac:dyDescent="0.4">
+      <c r="A68" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="B68" s="2"/>
+      <c r="C68" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D68" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E68" s="4"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A69" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B69" s="2"/>
+      <c r="C69" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D69" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E69" s="4"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A70" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B70" s="2"/>
+      <c r="C70" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D70" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E70" s="4"/>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A71" s="1"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E71" s="4"/>
+    </row>
+    <row r="72" spans="1:5" ht="16" x14ac:dyDescent="0.4">
+      <c r="A72" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B72" s="2"/>
+      <c r="C72" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E72" s="4"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A73" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B73" s="2"/>
+      <c r="C73" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E73" s="4"/>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A74" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B74" s="2"/>
+      <c r="C74" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E74" s="4"/>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A75" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B75" s="2"/>
+      <c r="C75" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D75" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E75" s="4"/>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A76" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B76" s="2"/>
+      <c r="C76" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D76" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E76" s="4"/>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A77" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B77" s="2"/>
+      <c r="C77" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D77" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E77" s="4"/>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A78" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B78" s="2"/>
+      <c r="C78" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D78" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E78" s="4"/>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A79" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B79" s="2"/>
+      <c r="C79" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D79" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E79" s="4"/>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A80" s="1"/>
+      <c r="B80" s="2"/>
+      <c r="C80" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D80" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E80" s="4"/>
+    </row>
+    <row r="81" spans="1:5" ht="16" x14ac:dyDescent="0.4">
+      <c r="A81" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="B81" s="2"/>
+      <c r="C81" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D81" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E81" s="4"/>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A82" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B82" s="2"/>
+      <c r="C82" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D82" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E82" s="4"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A83" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B83" s="2"/>
+      <c r="C83" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D83" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E83" s="4"/>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A84" s="1"/>
+      <c r="B84" s="2"/>
+      <c r="C84" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D84" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E84" s="4"/>
+    </row>
+    <row r="85" spans="1:5" ht="16" x14ac:dyDescent="0.4">
+      <c r="A85" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="B85" s="2"/>
+      <c r="C85" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D85" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E85" s="4"/>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A86" s="1"/>
+      <c r="B86" s="2"/>
+      <c r="C86" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D86" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E86" s="4"/>
+    </row>
+    <row r="87" spans="1:5" ht="16" x14ac:dyDescent="0.4">
+      <c r="A87" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="B87" s="2"/>
+      <c r="C87" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D87" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E87" s="4"/>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A88" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B88" s="2"/>
+      <c r="C88" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D88" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E88" s="4"/>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A89" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B89" s="2"/>
+      <c r="C89" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D89" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E89" s="4"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A90" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B90" s="2"/>
+      <c r="C90" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D90" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E90" s="4"/>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A91" s="1"/>
+      <c r="B91" s="2"/>
+      <c r="C91" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D91" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E91" s="4"/>
+    </row>
+    <row r="92" spans="1:5" ht="16" x14ac:dyDescent="0.4">
+      <c r="A92" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="B92" s="2"/>
+      <c r="C92" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D92" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E92" s="4"/>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A93" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B93" s="2"/>
+      <c r="C93" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D93" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E93" s="4"/>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A94" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B94" s="2"/>
+      <c r="C94" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D94" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E94" s="4"/>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A95" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B95" s="2"/>
+      <c r="C95" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D95" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E95" s="4"/>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A96" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B96" s="2"/>
+      <c r="C96" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D96" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E96" s="4"/>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A97" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B97" s="2"/>
+      <c r="C97" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D97" s="3">
+        <v>46139</v>
+      </c>
+      <c r="E97" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C38" xr:uid="{52EB43A6-14F6-40EB-BF81-7B4B1A3DB339}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C97" xr:uid="{52EB43A6-14F6-40EB-BF81-7B4B1A3DB339}">
       <formula1>$N$4:$N$10</formula1>
     </dataValidation>
   </dataValidations>
@@ -1551,71 +2318,68 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{191B8D4A-CCE5-43A3-8715-35D42E8F0862}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.26953125" customWidth="1"/>
     <col min="2" max="2" width="39.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="22" customFormat="1" ht="24" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="32" t="s">
+    <row r="1" spans="1:2" s="21" customFormat="1" ht="24" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A1" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="30" t="s">
+      <c r="B1" s="31"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="29" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="23" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="29" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="23" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="29" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="24" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="29" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="24" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="29" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="24" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="29" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B9" s="10"/>
     </row>
   </sheetData>

</xml_diff>